<commit_message>
thông tin thay đổi
</commit_message>
<xml_diff>
--- a/HNG_3_20250824/Metadata_3.xlsx
+++ b/HNG_3_20250824/Metadata_3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\XN\du-an-dung-chung\HNG_3_20250824\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13F2583F-8125-4AB0-B198-8B16A341D691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71D06E39-9C74-4FE6-B799-472632E4EC5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Thông tin lâm sàng" sheetId="3" r:id="rId1"/>
@@ -88,7 +88,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3043" uniqueCount="1069">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3045" uniqueCount="1070">
   <si>
     <t>https://docs.google.com/spreadsheets/d/1NL7nC96f90uNMKbf-Ps6YFaXbIP6V2Tgs1NXlk_JFB8/edit?gid=0#gid=0</t>
   </si>
@@ -3298,6 +3298,9 @@
   </si>
   <si>
     <t>TỔNG</t>
+  </si>
+  <si>
+    <t>%</t>
   </si>
 </sst>
 </file>
@@ -20125,8 +20128,14 @@
       <c r="C2" t="s">
         <v>1063</v>
       </c>
+      <c r="D2" s="69" t="s">
+        <v>1069</v>
+      </c>
       <c r="E2" t="s">
         <v>1067</v>
+      </c>
+      <c r="F2" s="69" t="s">
+        <v>1069</v>
       </c>
     </row>
     <row r="3" spans="2:15" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">

</xml_diff>